<commit_message>
New run, this time using ensemble with 5 models
</commit_message>
<xml_diff>
--- a/Code/results_Matthew.xlsx
+++ b/Code/results_Matthew.xlsx
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="134">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="151">
@@ -4290,7 +4290,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="175">
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194">
@@ -5315,7 +5315,7 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="197">
@@ -5865,7 +5865,7 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
@@ -6190,7 +6190,7 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="232">
@@ -6290,7 +6290,7 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236">
@@ -6390,7 +6390,7 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="240">
@@ -6515,7 +6515,7 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245">
@@ -7190,7 +7190,7 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="272">
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="280">
@@ -8065,7 +8065,7 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="307">
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="331">
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="E374" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="375">
@@ -11365,7 +11365,7 @@
         </is>
       </c>
       <c r="E438" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="439">
@@ -12740,7 +12740,7 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="494">
@@ -12890,7 +12890,7 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="500">
@@ -13240,7 +13240,7 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="514">
@@ -13365,7 +13365,7 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="519">
@@ -13690,7 +13690,7 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="532">
@@ -13990,7 +13990,7 @@
         </is>
       </c>
       <c r="E543" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="544">
@@ -14190,7 +14190,7 @@
         </is>
       </c>
       <c r="E551" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="552">
@@ -14415,7 +14415,7 @@
         </is>
       </c>
       <c r="E560" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="561">
@@ -14540,7 +14540,7 @@
         </is>
       </c>
       <c r="E565" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="566">
@@ -15590,7 +15590,7 @@
         </is>
       </c>
       <c r="E607" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="608">
@@ -15640,7 +15640,7 @@
         </is>
       </c>
       <c r="E609" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="610">
@@ -16665,7 +16665,7 @@
         </is>
       </c>
       <c r="E650" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="651">
@@ -16690,7 +16690,7 @@
         </is>
       </c>
       <c r="E651" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="652">
@@ -16765,7 +16765,7 @@
         </is>
       </c>
       <c r="E654" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="655">
@@ -17040,7 +17040,7 @@
         </is>
       </c>
       <c r="E665" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="666">
@@ -17390,7 +17390,7 @@
         </is>
       </c>
       <c r="E679" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="680">
@@ -17590,7 +17590,7 @@
         </is>
       </c>
       <c r="E687" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="688">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="E690" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="691">
@@ -17765,7 +17765,7 @@
         </is>
       </c>
       <c r="E694" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="695">
@@ -18715,7 +18715,7 @@
         </is>
       </c>
       <c r="E732" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="733">
@@ -18815,7 +18815,7 @@
         </is>
       </c>
       <c r="E736" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="737">
@@ -19265,7 +19265,7 @@
         </is>
       </c>
       <c r="E754" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="755">
@@ -19440,7 +19440,7 @@
         </is>
       </c>
       <c r="E761" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="762">
@@ -19765,7 +19765,7 @@
         </is>
       </c>
       <c r="E774" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="775">
@@ -19815,7 +19815,7 @@
         </is>
       </c>
       <c r="E776" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="777">
@@ -20715,7 +20715,7 @@
         </is>
       </c>
       <c r="E812" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="813">
@@ -20740,7 +20740,7 @@
         </is>
       </c>
       <c r="E813" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="814">
@@ -20790,7 +20790,7 @@
         </is>
       </c>
       <c r="E815" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="816">
@@ -20840,7 +20840,7 @@
         </is>
       </c>
       <c r="E817" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="818">
@@ -20940,7 +20940,7 @@
         </is>
       </c>
       <c r="E821" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="822">
@@ -21140,7 +21140,7 @@
         </is>
       </c>
       <c r="E829" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="830">
@@ -21315,7 +21315,7 @@
         </is>
       </c>
       <c r="E836" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="837">
@@ -21465,7 +21465,7 @@
         </is>
       </c>
       <c r="E842" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="843">
@@ -21690,7 +21690,7 @@
         </is>
       </c>
       <c r="E851" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="852">
@@ -22815,7 +22815,7 @@
         </is>
       </c>
       <c r="E896" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="897">
@@ -22890,7 +22890,7 @@
         </is>
       </c>
       <c r="E899" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="900">
@@ -23715,7 +23715,7 @@
         </is>
       </c>
       <c r="E932" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="933">
@@ -23915,7 +23915,7 @@
         </is>
       </c>
       <c r="E940" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="941">
@@ -23990,7 +23990,7 @@
         </is>
       </c>
       <c r="E943" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="944">
@@ -24490,7 +24490,7 @@
         </is>
       </c>
       <c r="E963" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="964">
@@ -24615,7 +24615,7 @@
         </is>
       </c>
       <c r="E968" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="969">
@@ -24690,7 +24690,7 @@
         </is>
       </c>
       <c r="E971" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="972">
@@ -24765,7 +24765,7 @@
         </is>
       </c>
       <c r="E974" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="975">
@@ -24965,7 +24965,7 @@
         </is>
       </c>
       <c r="E982" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="983">
@@ -25015,7 +25015,7 @@
         </is>
       </c>
       <c r="E984" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="985">
@@ -25215,7 +25215,7 @@
         </is>
       </c>
       <c r="E992" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="993">
@@ -25415,7 +25415,7 @@
         </is>
       </c>
       <c r="E1000" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1001">
@@ -25540,7 +25540,7 @@
         </is>
       </c>
       <c r="E1005" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1006">
@@ -26065,7 +26065,7 @@
         </is>
       </c>
       <c r="E1026" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1027">
@@ -26315,7 +26315,7 @@
         </is>
       </c>
       <c r="E1036" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1037">
@@ -26590,7 +26590,7 @@
         </is>
       </c>
       <c r="E1047" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1048">
@@ -26690,7 +26690,7 @@
         </is>
       </c>
       <c r="E1051" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1052">
@@ -26915,7 +26915,7 @@
         </is>
       </c>
       <c r="E1060" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1061">
@@ -27190,7 +27190,7 @@
         </is>
       </c>
       <c r="E1071" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1072">
@@ -27390,7 +27390,7 @@
         </is>
       </c>
       <c r="E1079" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1080">
@@ -27565,7 +27565,7 @@
         </is>
       </c>
       <c r="E1086" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1087">
@@ -28190,7 +28190,7 @@
         </is>
       </c>
       <c r="E1111" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1112">
@@ -28990,7 +28990,7 @@
         </is>
       </c>
       <c r="E1143" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1144">
@@ -29165,7 +29165,7 @@
         </is>
       </c>
       <c r="E1150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1151">
@@ -29290,7 +29290,7 @@
         </is>
       </c>
       <c r="E1155" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1156">
@@ -29315,7 +29315,7 @@
         </is>
       </c>
       <c r="E1156" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1157">
@@ -29840,7 +29840,7 @@
         </is>
       </c>
       <c r="E1177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1178">
@@ -30015,7 +30015,7 @@
         </is>
       </c>
       <c r="E1184" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1185">
@@ -30665,7 +30665,7 @@
         </is>
       </c>
       <c r="E1210" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1211">
@@ -30815,7 +30815,7 @@
         </is>
       </c>
       <c r="E1216" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1217">
@@ -31015,7 +31015,7 @@
         </is>
       </c>
       <c r="E1224" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1225">
@@ -31190,7 +31190,7 @@
         </is>
       </c>
       <c r="E1231" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1232">
@@ -31315,7 +31315,7 @@
         </is>
       </c>
       <c r="E1236" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1237">
@@ -31390,7 +31390,7 @@
         </is>
       </c>
       <c r="E1239" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1240">
@@ -31490,7 +31490,7 @@
         </is>
       </c>
       <c r="E1243" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1244">
@@ -31640,7 +31640,7 @@
         </is>
       </c>
       <c r="E1249" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1250">
@@ -31815,7 +31815,7 @@
         </is>
       </c>
       <c r="E1256" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1257">
@@ -31840,7 +31840,7 @@
         </is>
       </c>
       <c r="E1257" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1258">
@@ -31890,7 +31890,7 @@
         </is>
       </c>
       <c r="E1259" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1260">
@@ -32040,7 +32040,7 @@
         </is>
       </c>
       <c r="E1265" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1266">
@@ -32240,7 +32240,7 @@
         </is>
       </c>
       <c r="E1273" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1274">
@@ -32265,7 +32265,7 @@
         </is>
       </c>
       <c r="E1274" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1275">
@@ -32740,7 +32740,7 @@
         </is>
       </c>
       <c r="E1293" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1294">
@@ -32865,7 +32865,7 @@
         </is>
       </c>
       <c r="E1298" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1299">
@@ -32915,7 +32915,7 @@
         </is>
       </c>
       <c r="E1300" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1301">
@@ -33240,7 +33240,7 @@
         </is>
       </c>
       <c r="E1313" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1314">
@@ -33290,7 +33290,7 @@
         </is>
       </c>
       <c r="E1315" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1316">
@@ -33340,7 +33340,7 @@
         </is>
       </c>
       <c r="E1317" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1318">
@@ -33590,7 +33590,7 @@
         </is>
       </c>
       <c r="E1327" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1328">
@@ -34215,7 +34215,7 @@
         </is>
       </c>
       <c r="E1352" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1353">
@@ -34265,7 +34265,7 @@
         </is>
       </c>
       <c r="E1354" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1355">
@@ -34565,7 +34565,7 @@
         </is>
       </c>
       <c r="E1366" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1367">
@@ -34715,7 +34715,7 @@
         </is>
       </c>
       <c r="E1372" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1373">
@@ -34940,7 +34940,7 @@
         </is>
       </c>
       <c r="E1381" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1382">
@@ -35040,7 +35040,7 @@
         </is>
       </c>
       <c r="E1385" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1386">
@@ -35265,7 +35265,7 @@
         </is>
       </c>
       <c r="E1394" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1395">
@@ -35915,7 +35915,7 @@
         </is>
       </c>
       <c r="E1420" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1421">
@@ -36290,7 +36290,7 @@
         </is>
       </c>
       <c r="E1435" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1436">
@@ -36815,7 +36815,7 @@
         </is>
       </c>
       <c r="E1456" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1457">
@@ -37390,7 +37390,7 @@
         </is>
       </c>
       <c r="E1479" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1480">
@@ -37465,7 +37465,7 @@
         </is>
       </c>
       <c r="E1482" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1483">
@@ -37565,7 +37565,7 @@
         </is>
       </c>
       <c r="E1486" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1487">
@@ -38390,7 +38390,7 @@
         </is>
       </c>
       <c r="E1519" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1520">
@@ -38415,7 +38415,7 @@
         </is>
       </c>
       <c r="E1520" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1521">
@@ -39615,7 +39615,7 @@
         </is>
       </c>
       <c r="E1568" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1569">
@@ -39640,7 +39640,7 @@
         </is>
       </c>
       <c r="E1569" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1570">
@@ -39965,7 +39965,7 @@
         </is>
       </c>
       <c r="E1582" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1583">
@@ -40640,7 +40640,7 @@
         </is>
       </c>
       <c r="E1609" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1610">
@@ -40865,7 +40865,7 @@
         </is>
       </c>
       <c r="E1618" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1619">
@@ -40890,7 +40890,7 @@
         </is>
       </c>
       <c r="E1619" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1620">
@@ -40915,7 +40915,7 @@
         </is>
       </c>
       <c r="E1620" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1621">
@@ -41040,7 +41040,7 @@
         </is>
       </c>
       <c r="E1625" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1626">
@@ -41265,7 +41265,7 @@
         </is>
       </c>
       <c r="E1634" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1635">
@@ -41540,7 +41540,7 @@
         </is>
       </c>
       <c r="E1645" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1646">
@@ -41590,7 +41590,7 @@
         </is>
       </c>
       <c r="E1647" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1648">
@@ -41765,7 +41765,7 @@
         </is>
       </c>
       <c r="E1654" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1655">
@@ -41890,7 +41890,7 @@
         </is>
       </c>
       <c r="E1659" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1660">
@@ -42065,7 +42065,7 @@
         </is>
       </c>
       <c r="E1666" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1667">
@@ -42140,7 +42140,7 @@
         </is>
       </c>
       <c r="E1669" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1670">
@@ -42315,7 +42315,7 @@
         </is>
       </c>
       <c r="E1676" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1677">
@@ -42865,7 +42865,7 @@
         </is>
       </c>
       <c r="E1698" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1699">
@@ -43715,7 +43715,7 @@
         </is>
       </c>
       <c r="E1732" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1733">
@@ -44190,7 +44190,7 @@
         </is>
       </c>
       <c r="E1751" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1752">
@@ -44390,7 +44390,7 @@
         </is>
       </c>
       <c r="E1759" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1760">
@@ -44690,7 +44690,7 @@
         </is>
       </c>
       <c r="E1771" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1772">
@@ -44865,7 +44865,7 @@
         </is>
       </c>
       <c r="E1778" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1779">
@@ -45015,7 +45015,7 @@
         </is>
       </c>
       <c r="E1784" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1785">
@@ -45465,7 +45465,7 @@
         </is>
       </c>
       <c r="E1802" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1803">
@@ -45515,7 +45515,7 @@
         </is>
       </c>
       <c r="E1804" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1805">
@@ -45590,7 +45590,7 @@
         </is>
       </c>
       <c r="E1807" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1808">
@@ -45740,7 +45740,7 @@
         </is>
       </c>
       <c r="E1813" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1814">
@@ -45840,7 +45840,7 @@
         </is>
       </c>
       <c r="E1817" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1818">
@@ -45940,7 +45940,7 @@
         </is>
       </c>
       <c r="E1821" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1822">
@@ -46265,7 +46265,7 @@
         </is>
       </c>
       <c r="E1834" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1835">
@@ -46365,7 +46365,7 @@
         </is>
       </c>
       <c r="E1838" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1839">
@@ -46465,7 +46465,7 @@
         </is>
       </c>
       <c r="E1842" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1843">
@@ -47390,7 +47390,7 @@
         </is>
       </c>
       <c r="E1879" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1880">
@@ -47565,7 +47565,7 @@
         </is>
       </c>
       <c r="E1886" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1887">
@@ -47915,7 +47915,7 @@
         </is>
       </c>
       <c r="E1900" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1901">
@@ -48815,7 +48815,7 @@
         </is>
       </c>
       <c r="E1936" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1937">
@@ -49065,7 +49065,7 @@
         </is>
       </c>
       <c r="E1946" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1947">
@@ -49590,7 +49590,7 @@
         </is>
       </c>
       <c r="E1967" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1968">
@@ -50665,7 +50665,7 @@
         </is>
       </c>
       <c r="E2010" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2011">
@@ -51065,7 +51065,7 @@
         </is>
       </c>
       <c r="E2026" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2027">
@@ -51190,7 +51190,7 @@
         </is>
       </c>
       <c r="E2031" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2032">
@@ -51215,7 +51215,7 @@
         </is>
       </c>
       <c r="E2032" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2033">
@@ -51390,7 +51390,7 @@
         </is>
       </c>
       <c r="E2039" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2040">
@@ -51665,7 +51665,7 @@
         </is>
       </c>
       <c r="E2050" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2051">
@@ -52115,7 +52115,7 @@
         </is>
       </c>
       <c r="E2068" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2069">
@@ -52915,7 +52915,7 @@
         </is>
       </c>
       <c r="E2100" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2101">
@@ -53290,7 +53290,7 @@
         </is>
       </c>
       <c r="E2115" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2116">
@@ -53390,7 +53390,7 @@
         </is>
       </c>
       <c r="E2119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2120">
@@ -53515,7 +53515,7 @@
         </is>
       </c>
       <c r="E2124" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2125">
@@ -53590,7 +53590,7 @@
         </is>
       </c>
       <c r="E2127" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2128">
@@ -53665,7 +53665,7 @@
         </is>
       </c>
       <c r="E2130" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2131">
@@ -54215,7 +54215,7 @@
         </is>
       </c>
       <c r="E2152" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2153">
@@ -54365,7 +54365,7 @@
         </is>
       </c>
       <c r="E2158" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2159">
@@ -55040,7 +55040,7 @@
         </is>
       </c>
       <c r="E2185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2186">
@@ -55065,7 +55065,7 @@
         </is>
       </c>
       <c r="E2186" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2187">
@@ -56065,7 +56065,7 @@
         </is>
       </c>
       <c r="E2226" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2227">
@@ -56215,7 +56215,7 @@
         </is>
       </c>
       <c r="E2232" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2233">
@@ -56815,7 +56815,7 @@
         </is>
       </c>
       <c r="E2256" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2257">
@@ -56990,7 +56990,7 @@
         </is>
       </c>
       <c r="E2263" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2264">
@@ -57640,7 +57640,7 @@
         </is>
       </c>
       <c r="E2289" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2290">
@@ -57840,7 +57840,7 @@
         </is>
       </c>
       <c r="E2297" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2298">
@@ -58240,7 +58240,7 @@
         </is>
       </c>
       <c r="E2313" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2314">
@@ -58415,7 +58415,7 @@
         </is>
       </c>
       <c r="E2320" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2321">
@@ -58640,7 +58640,7 @@
         </is>
       </c>
       <c r="E2329" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2330">
@@ -59215,7 +59215,7 @@
         </is>
       </c>
       <c r="E2352" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2353">
@@ -59390,7 +59390,7 @@
         </is>
       </c>
       <c r="E2359" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2360">
@@ -59415,7 +59415,7 @@
         </is>
       </c>
       <c r="E2360" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2361">
@@ -59790,7 +59790,7 @@
         </is>
       </c>
       <c r="E2375" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2376">
@@ -60340,7 +60340,7 @@
         </is>
       </c>
       <c r="E2397" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2398">
@@ -60840,7 +60840,7 @@
         </is>
       </c>
       <c r="E2417" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2418">
@@ -60890,7 +60890,7 @@
         </is>
       </c>
       <c r="E2419" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2420">
@@ -61115,7 +61115,7 @@
         </is>
       </c>
       <c r="E2428" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2429">
@@ -61165,7 +61165,7 @@
         </is>
       </c>
       <c r="E2430" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2431">
@@ -61390,7 +61390,7 @@
         </is>
       </c>
       <c r="E2439" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2440">
@@ -61665,7 +61665,7 @@
         </is>
       </c>
       <c r="E2450" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2451">
@@ -62065,7 +62065,7 @@
         </is>
       </c>
       <c r="E2466" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2467">
@@ -62390,7 +62390,7 @@
         </is>
       </c>
       <c r="E2479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2480">
@@ -62665,7 +62665,7 @@
         </is>
       </c>
       <c r="E2490" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2491">
@@ -63190,7 +63190,7 @@
         </is>
       </c>
       <c r="E2511" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2512">
@@ -64290,7 +64290,7 @@
         </is>
       </c>
       <c r="E2555" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2556">
@@ -64390,7 +64390,7 @@
         </is>
       </c>
       <c r="E2559" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2560">
@@ -64415,7 +64415,7 @@
         </is>
       </c>
       <c r="E2560" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2561">
@@ -64990,7 +64990,7 @@
         </is>
       </c>
       <c r="E2583" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2584">
@@ -65015,7 +65015,7 @@
         </is>
       </c>
       <c r="E2584" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2585">
@@ -65190,7 +65190,7 @@
         </is>
       </c>
       <c r="E2591" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2592">

</xml_diff>